<commit_message>
Complications des actes : thème du MCO, code S% ramené à un code
Le classeur est destiné au MCO : le thème quitte le SMR. La cellule
« S% de lésion superficielle ou T14.0 si la localisation n'est pas
précisée » de la colonne des codes devient « S% ou T14.0 », sa précision
passe en proposition de code plus précis ; la colonne des codes retombe
de 700 à 172 px.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011pkvaUPcVJWMQggb4SNT9K
</commit_message>
<xml_diff>
--- a/data/complications/liste_code_complications.xlsx
+++ b/data/complications/liste_code_complications.xlsx
@@ -9574,7 +9574,7 @@
       </c>
       <c r="B306" s="104" t="inlineStr">
         <is>
-          <t>S% de lésion superficielle ou T14.0 si la localisation n'est pas précisée</t>
+          <t>S% ou T14.0</t>
         </is>
       </c>
       <c r="C306" s="1" t="n"/>
@@ -9588,7 +9588,11 @@
           <t xml:space="preserve">T81.8 + code Y </t>
         </is>
       </c>
-      <c r="F306" s="11" t="n"/>
+      <c r="F306" s="11" t="inlineStr">
+        <is>
+          <t>S% de lésion superficielle ; T14.0 si la localisation n'est pas précisée</t>
+        </is>
+      </c>
       <c r="G306" s="6" t="n"/>
     </row>
     <row r="307" ht="24" customHeight="1">

</xml_diff>

<commit_message>
Complications des actes : mise en forme du classeur, CMA code par code
- Classeur réédité depuis l'original en gardant le texte enrichi : les
  « à ne pas utiliser » en rouge et les CMA colorées perdus à la
  première édition sont de retour. « K28 .- » devient « K28.- ».
- Une cellule de plusieurs codes (« L08.8 ou L08.0 », « G62.8 +G72.8 »)
  prend le niveau de CMA de chacun de ses codes au lieu de rester vide ;
  la note de la page le dit, et nomme aussi les codes non terminaux.
- Le champ des codes Y n'affiche plus le raccourci « / », qui mène au
  premier champ de la page.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011pkvaUPcVJWMQggb4SNT9K
</commit_message>
<xml_diff>
--- a/data/complications/liste_code_complications.xlsx
+++ b/data/complications/liste_code_complications.xlsx
@@ -1156,7 +1156,19 @@
       </c>
       <c r="C2" s="53" t="inlineStr">
         <is>
-          <t>❹ SSR</t>
+          <r>
+            <t>❹</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="9" tint="-0.249977111117893"/>
+              <sz val="9"/>
+            </rPr>
+            <t xml:space="preserve"> SSR</t>
+          </r>
         </is>
       </c>
       <c r="D2" s="1" t="inlineStr">
@@ -1482,8 +1494,20 @@
       <c r="C14" s="123" t="n"/>
       <c r="D14" s="124" t="inlineStr">
         <is>
-          <t>Code de fin de chapitre 
-IMPRECIS à ne pas utiliser</t>
+          <r>
+            <t xml:space="preserve">Code de fin de chapitre 
+IMPRECIS </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color rgb="FFFF0000"/>
+              <sz val="9"/>
+              <scheme val="minor"/>
+            </rPr>
+            <t>à ne pas utiliser</t>
+          </r>
         </is>
       </c>
       <c r="E14" s="125" t="inlineStr">
@@ -1508,8 +1532,20 @@
       <c r="C15" s="123" t="n"/>
       <c r="D15" s="124" t="inlineStr">
         <is>
-          <t>Code de fin de chapitre 
-IMPRECIS à ne pas utiliser et interdit en DP</t>
+          <r>
+            <t xml:space="preserve">Code de fin de chapitre 
+IMPRECIS </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color rgb="FFFF0000"/>
+              <sz val="9"/>
+              <scheme val="minor"/>
+            </rPr>
+            <t>à ne pas utiliser et interdit en DP</t>
+          </r>
         </is>
       </c>
       <c r="E15" s="125" t="inlineStr">
@@ -1543,7 +1579,28 @@
       </c>
       <c r="E16" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Code T81.8 ❷  + code Y </t>
+          <r>
+            <t xml:space="preserve">Code T81.8 </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color rgb="FF0070C0"/>
+              <sz val="9"/>
+              <scheme val="minor"/>
+            </rPr>
+            <t>❷</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <sz val="9"/>
+              <scheme val="minor"/>
+            </rPr>
+            <t xml:space="preserve">  + code Y </t>
+          </r>
         </is>
       </c>
       <c r="F16" s="11" t="n"/>
@@ -1884,8 +1941,20 @@
       <c r="C28" s="123" t="n"/>
       <c r="D28" s="124" t="inlineStr">
         <is>
-          <t>Code de fin de chapitre 
-IMPRECIS à ne pas utiliser et interdit en DP</t>
+          <r>
+            <t xml:space="preserve">Code de fin de chapitre 
+IMPRECIS </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color rgb="FFFF0000"/>
+              <sz val="9"/>
+              <scheme val="minor"/>
+            </rPr>
+            <t>à ne pas utiliser et interdit en DP</t>
+          </r>
         </is>
       </c>
       <c r="E28" s="125" t="inlineStr">
@@ -1988,8 +2057,20 @@
       <c r="C32" s="124" t="n"/>
       <c r="D32" s="124" t="inlineStr">
         <is>
-          <t>Code de fin de chapitre 
-IMPRECIS à ne pas utiliser</t>
+          <r>
+            <t xml:space="preserve">Code de fin de chapitre 
+IMPRECIS </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color rgb="FFFF0000"/>
+              <sz val="9"/>
+              <scheme val="minor"/>
+            </rPr>
+            <t>à ne pas utiliser</t>
+          </r>
         </is>
       </c>
       <c r="E32" s="125" t="inlineStr">
@@ -2014,8 +2095,20 @@
       <c r="C33" s="123" t="n"/>
       <c r="D33" s="124" t="inlineStr">
         <is>
-          <t>Code de fin de chapitre 
-IMPRECIS à ne pas utiliser et interdit en DP</t>
+          <r>
+            <t xml:space="preserve">Code de fin de chapitre 
+IMPRECIS </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color rgb="FFFF0000"/>
+              <sz val="9"/>
+              <scheme val="minor"/>
+            </rPr>
+            <t>à ne pas utiliser et interdit en DP</t>
+          </r>
         </is>
       </c>
       <c r="E33" s="125" t="inlineStr">
@@ -2097,8 +2190,20 @@
       <c r="C36" s="123" t="n"/>
       <c r="D36" s="124" t="inlineStr">
         <is>
-          <t>Code de fin de chapitre 
-IMPRECIS à ne pas utiliser</t>
+          <r>
+            <t xml:space="preserve">Code de fin de chapitre 
+IMPRECIS </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color rgb="FFFF0000"/>
+              <sz val="9"/>
+              <scheme val="minor"/>
+            </rPr>
+            <t>à ne pas utiliser</t>
+          </r>
         </is>
       </c>
       <c r="E36" s="125" t="inlineStr">
@@ -2123,8 +2228,20 @@
       <c r="C37" s="123" t="n"/>
       <c r="D37" s="124" t="inlineStr">
         <is>
-          <t>Code de fin de chapitre 
-IMPRECIS à ne pas utiliser et interdit en DP</t>
+          <r>
+            <t xml:space="preserve">Code de fin de chapitre 
+IMPRECIS </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color rgb="FFFF0000"/>
+              <sz val="9"/>
+              <scheme val="minor"/>
+            </rPr>
+            <t>à ne pas utiliser et interdit en DP</t>
+          </r>
         </is>
       </c>
       <c r="E37" s="125" t="inlineStr">
@@ -2181,7 +2298,26 @@
       </c>
       <c r="C39" s="55" t="inlineStr">
         <is>
-          <t>❸ ou ❹</t>
+          <r>
+            <t xml:space="preserve">❸ </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri Light"/>
+              <family val="2"/>
+              <sz val="9"/>
+            </rPr>
+            <t>ou</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri Light"/>
+              <family val="2"/>
+              <color rgb="FFFF0000"/>
+              <sz val="9"/>
+            </rPr>
+            <t xml:space="preserve"> ❹</t>
+          </r>
         </is>
       </c>
       <c r="D39" s="1" t="inlineStr">
@@ -2675,8 +2811,20 @@
       <c r="C55" s="124" t="n"/>
       <c r="D55" s="124" t="inlineStr">
         <is>
-          <t>Code de fin de chapitre 
-IMPRECIS à ne pas utiliser</t>
+          <r>
+            <t xml:space="preserve">Code de fin de chapitre 
+IMPRECIS </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color rgb="FFFF0000"/>
+              <sz val="9"/>
+              <scheme val="minor"/>
+            </rPr>
+            <t>à ne pas utiliser</t>
+          </r>
         </is>
       </c>
       <c r="E55" s="125" t="inlineStr">
@@ -2705,8 +2853,20 @@
       <c r="C56" s="123" t="n"/>
       <c r="D56" s="124" t="inlineStr">
         <is>
-          <t>Code de fin de chapitre 
-IMPRECIS à ne pas utiliser et interdit en DP</t>
+          <r>
+            <t xml:space="preserve">Code de fin de chapitre 
+IMPRECIS </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color rgb="FFFF0000"/>
+              <sz val="9"/>
+              <scheme val="minor"/>
+            </rPr>
+            <t>à ne pas utiliser et interdit en DP</t>
+          </r>
         </is>
       </c>
       <c r="E56" s="125" t="inlineStr">
@@ -2730,7 +2890,56 @@
       </c>
       <c r="C57" s="4" t="inlineStr">
         <is>
-          <t>❷ ou ❸ ou ❹</t>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color rgb="FF0070C0"/>
+              <sz val="9"/>
+              <scheme val="minor"/>
+            </rPr>
+            <t>❷</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="9"/>
+              <scheme val="minor"/>
+            </rPr>
+            <t xml:space="preserve"> ou </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color rgb="FFFFC000"/>
+              <sz val="9"/>
+              <scheme val="minor"/>
+            </rPr>
+            <t>❸</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="9"/>
+              <scheme val="minor"/>
+            </rPr>
+            <t xml:space="preserve"> ou </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color rgb="FFFF0000"/>
+              <sz val="9"/>
+              <scheme val="minor"/>
+            </rPr>
+            <t>❹</t>
+          </r>
         </is>
       </c>
       <c r="D57" s="1" t="inlineStr">
@@ -2904,7 +3113,24 @@
       </c>
       <c r="C63" s="57" t="inlineStr">
         <is>
-          <t>❹  SSR</t>
+          <r>
+            <rPr>
+              <rFont val="Calibri Light"/>
+              <family val="2"/>
+              <color rgb="FFFF0000"/>
+              <sz val="9"/>
+            </rPr>
+            <t xml:space="preserve">❹  </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri Light"/>
+              <family val="2"/>
+              <color rgb="FF00B050"/>
+              <sz val="9"/>
+            </rPr>
+            <t>SSR</t>
+          </r>
         </is>
       </c>
       <c r="D63" s="1" t="inlineStr">
@@ -3116,8 +3342,20 @@
       <c r="C70" s="123" t="n"/>
       <c r="D70" s="124" t="inlineStr">
         <is>
-          <t>Code de fin de chapitre 
-IMPRECIS à ne pas utiliser</t>
+          <r>
+            <t xml:space="preserve">Code de fin de chapitre 
+IMPRECIS </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color rgb="FFFF0000"/>
+              <sz val="9"/>
+              <scheme val="minor"/>
+            </rPr>
+            <t>à ne pas utiliser</t>
+          </r>
         </is>
       </c>
       <c r="E70" s="125" t="inlineStr">
@@ -3149,8 +3387,20 @@
       <c r="C71" s="123" t="n"/>
       <c r="D71" s="124" t="inlineStr">
         <is>
-          <t>Code de fin de chapitre 
-IMPRECIS à ne pas utiliser et interdit en DP</t>
+          <r>
+            <t xml:space="preserve">Code de fin de chapitre 
+IMPRECIS </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color rgb="FFFF0000"/>
+              <sz val="9"/>
+              <scheme val="minor"/>
+            </rPr>
+            <t>à ne pas utiliser et interdit en DP</t>
+          </r>
         </is>
       </c>
       <c r="E71" s="125" t="inlineStr">
@@ -3251,7 +3501,19 @@
     <row r="75">
       <c r="A75" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Oesophagite radique </t>
+          <r>
+            <t>Oesophagite radique</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color rgb="FF00B0F0"/>
+              <sz val="9"/>
+              <scheme val="minor"/>
+            </rPr>
+            <t> </t>
+          </r>
         </is>
       </c>
       <c r="B75" s="10" t="inlineStr">
@@ -3294,7 +3556,56 @@
       </c>
       <c r="C76" s="4" t="inlineStr">
         <is>
-          <t>❷ ou ❸ ou ❹</t>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color rgb="FF0070C0"/>
+              <sz val="9"/>
+              <scheme val="minor"/>
+            </rPr>
+            <t>❷</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="9"/>
+              <scheme val="minor"/>
+            </rPr>
+            <t xml:space="preserve"> ou </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color rgb="FFFFC000"/>
+              <sz val="9"/>
+              <scheme val="minor"/>
+            </rPr>
+            <t>❸</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="9"/>
+              <scheme val="minor"/>
+            </rPr>
+            <t xml:space="preserve"> ou </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color rgb="FFFF0000"/>
+              <sz val="9"/>
+              <scheme val="minor"/>
+            </rPr>
+            <t>❹</t>
+          </r>
         </is>
       </c>
       <c r="D76" s="1" t="inlineStr">
@@ -3438,12 +3749,60 @@
       </c>
       <c r="B81" s="10" t="inlineStr">
         <is>
-          <t>K28 .-</t>
+          <t>K28.-</t>
         </is>
       </c>
       <c r="C81" s="4" t="inlineStr">
         <is>
-          <t>rien ou ❸ ou ❹</t>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <sz val="9"/>
+              <scheme val="minor"/>
+            </rPr>
+            <t>rien</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="9"/>
+              <scheme val="minor"/>
+            </rPr>
+            <t xml:space="preserve"> ou </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color rgb="FFFFC000"/>
+              <sz val="9"/>
+              <scheme val="minor"/>
+            </rPr>
+            <t>❸</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="9"/>
+              <scheme val="minor"/>
+            </rPr>
+            <t xml:space="preserve"> ou </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color rgb="FFFF0000"/>
+              <sz val="9"/>
+              <scheme val="minor"/>
+            </rPr>
+            <t>❹</t>
+          </r>
         </is>
       </c>
       <c r="D81" s="1" t="inlineStr">
@@ -3530,7 +3889,45 @@
       </c>
       <c r="C84" s="4" t="inlineStr">
         <is>
-          <t>Rien ou ❷ ou ❸</t>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <sz val="9"/>
+              <scheme val="minor"/>
+            </rPr>
+            <t xml:space="preserve">Rien ou </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color rgb="FF0070C0"/>
+              <sz val="9"/>
+              <scheme val="minor"/>
+            </rPr>
+            <t>❷</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="9"/>
+              <scheme val="minor"/>
+            </rPr>
+            <t xml:space="preserve"> ou </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color rgb="FFFFC000"/>
+              <sz val="9"/>
+              <scheme val="minor"/>
+            </rPr>
+            <t>❸</t>
+          </r>
         </is>
       </c>
       <c r="D84" s="4" t="inlineStr">
@@ -3912,8 +4309,52 @@
     <row r="97" ht="132" customHeight="1">
       <c r="A97" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mauvais résultats fonctionnels d’une colostomie et d’une entérostomie
+          <r>
+            <t xml:space="preserve">Mauvais résultats fonctionnels d’une </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="9"/>
+              <scheme val="minor"/>
+            </rPr>
+            <t>colostomie</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="9"/>
+              <scheme val="minor"/>
+            </rPr>
+            <t xml:space="preserve"> et d’une </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="9"/>
+              <scheme val="minor"/>
+            </rPr>
+            <t>entérostomie</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="9"/>
+              <scheme val="minor"/>
+            </rPr>
+            <t xml:space="preserve">
 ex : douleur ou saignement  ou prolapsus  ou sténose orifice ou difficultés d'adaptation des poches </t>
+          </r>
         </is>
       </c>
       <c r="B97" s="10" t="inlineStr">
@@ -3923,7 +4364,18 @@
       </c>
       <c r="C97" s="55" t="inlineStr">
         <is>
-          <t>❸ SSR</t>
+          <r>
+            <t xml:space="preserve">❸ </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri Light"/>
+              <family val="2"/>
+              <color rgb="FF00B050"/>
+              <sz val="9"/>
+            </rPr>
+            <t>SSR</t>
+          </r>
         </is>
       </c>
       <c r="D97" s="1" t="inlineStr">
@@ -3939,12 +4391,32 @@
       <c r="F97" s="11" t="n"/>
       <c r="G97" s="12" t="inlineStr">
         <is>
-          <t>Colostomies ou entérostomies
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="9"/>
+              <scheme val="minor"/>
+            </rPr>
+            <t>Colostomies ou entérostomies</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="9"/>
+              <scheme val="minor"/>
+            </rPr>
+            <t xml:space="preserve">
 douleurs stomie (AGORA 106523) 
 saignement stomie (AGORA 31146 et 21121) 
 prolapsus stomial (AGORA 116390)
 sténose orifice colostomie (AGORA 36998)
 difficultés d'adaption des poches de stomie (AGORA 171260)</t>
+          </r>
         </is>
       </c>
     </row>
@@ -3987,8 +4459,20 @@
       <c r="C99" s="123" t="n"/>
       <c r="D99" s="124" t="inlineStr">
         <is>
-          <t>Code de fin de chapitre 
-IMPRECIS à ne pas utiliser</t>
+          <r>
+            <t xml:space="preserve">Code de fin de chapitre 
+IMPRECIS </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color rgb="FFFF0000"/>
+              <sz val="9"/>
+              <scheme val="minor"/>
+            </rPr>
+            <t>à ne pas utiliser</t>
+          </r>
         </is>
       </c>
       <c r="E99" s="125" t="inlineStr">
@@ -4018,8 +4502,20 @@
       <c r="C100" s="123" t="n"/>
       <c r="D100" s="124" t="inlineStr">
         <is>
-          <t>Code de fin de chapitre 
-IMPRECIS à ne pas utiliser et interdit en DP</t>
+          <r>
+            <t xml:space="preserve">Code de fin de chapitre 
+IMPRECIS </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color rgb="FFFF0000"/>
+              <sz val="9"/>
+              <scheme val="minor"/>
+            </rPr>
+            <t>à ne pas utiliser et interdit en DP</t>
+          </r>
         </is>
       </c>
       <c r="E100" s="125" t="inlineStr">
@@ -4863,7 +5359,27 @@
       </c>
       <c r="E128" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Code T84.5❹  + code Y </t>
+          <r>
+            <t>Code T84.5</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color rgb="FFFF0000"/>
+              <sz val="9"/>
+            </rPr>
+            <t>❹</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <sz val="9"/>
+              <scheme val="minor"/>
+            </rPr>
+            <t xml:space="preserve">  + code Y </t>
+          </r>
         </is>
       </c>
       <c r="F128" s="11" t="n"/>
@@ -4944,7 +5460,19 @@
       </c>
       <c r="C131" s="54" t="inlineStr">
         <is>
-          <t>❷ SSR</t>
+          <r>
+            <t xml:space="preserve">❷ </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color rgb="FF00B050"/>
+              <sz val="9"/>
+              <scheme val="minor"/>
+            </rPr>
+            <t>SSR</t>
+          </r>
         </is>
       </c>
       <c r="D131" s="1" t="inlineStr">
@@ -5119,7 +5647,33 @@
       </c>
       <c r="C137" s="64" t="inlineStr">
         <is>
-          <t>❸ SSR</t>
+          <r>
+            <rPr>
+              <rFont val="Calibri Light"/>
+              <family val="2"/>
+              <color rgb="FFFFC000"/>
+              <sz val="9"/>
+            </rPr>
+            <t>❸</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri Light"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="9"/>
+            </rPr>
+            <t> </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color rgb="FF00B050"/>
+              <sz val="9"/>
+            </rPr>
+            <t>SSR</t>
+          </r>
         </is>
       </c>
       <c r="D137" s="1" t="inlineStr">
@@ -5153,8 +5707,20 @@
       <c r="C138" s="94" t="n"/>
       <c r="D138" s="94" t="inlineStr">
         <is>
-          <t>Code de fin de chapitre 
-IMPRECIS à ne pas utiliser</t>
+          <r>
+            <t xml:space="preserve">Code de fin de chapitre 
+IMPRECIS </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color rgb="FFFF0000"/>
+              <sz val="9"/>
+              <scheme val="minor"/>
+            </rPr>
+            <t>à ne pas utiliser</t>
+          </r>
         </is>
       </c>
       <c r="E138" s="95" t="inlineStr">
@@ -5179,8 +5745,20 @@
       <c r="C139" s="94" t="n"/>
       <c r="D139" s="94" t="inlineStr">
         <is>
-          <t>Code de fin de chapitre 
-IMPRECIS à ne pas utiliser et interdit en DP</t>
+          <r>
+            <t xml:space="preserve">Code de fin de chapitre 
+IMPRECIS </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color rgb="FFFF0000"/>
+              <sz val="9"/>
+              <scheme val="minor"/>
+            </rPr>
+            <t>à ne pas utiliser et interdit en DP</t>
+          </r>
         </is>
       </c>
       <c r="E139" s="95" t="inlineStr">
@@ -5194,7 +5772,30 @@
     <row r="140">
       <c r="A140" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Insuffisance rénale aigue IRA organique ou non précisée post opératoire </t>
+          <r>
+            <t xml:space="preserve">Insuffisance rénale aigue IRA </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="9"/>
+              <scheme val="minor"/>
+            </rPr>
+            <t>organique</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="9"/>
+              <scheme val="minor"/>
+            </rPr>
+            <t xml:space="preserve"> ou non précisée post opératoire </t>
+          </r>
         </is>
       </c>
       <c r="B140" s="10" t="inlineStr">
@@ -5223,7 +5824,30 @@
     <row r="141">
       <c r="A141" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Insuffisance rénale chronique IRC organique ou non précisée post opératoire </t>
+          <r>
+            <t xml:space="preserve">Insuffisance rénale chronique IRC </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="9"/>
+              <scheme val="minor"/>
+            </rPr>
+            <t>organique</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="9"/>
+              <scheme val="minor"/>
+            </rPr>
+            <t xml:space="preserve"> ou non précisée post opératoire </t>
+          </r>
         </is>
       </c>
       <c r="B141" s="10" t="inlineStr">
@@ -5595,8 +6219,20 @@
       </c>
       <c r="D154" s="94" t="inlineStr">
         <is>
-          <t xml:space="preserve">Code de Fin de chapitre à éviter 
+          <r>
+            <t xml:space="preserve">Code de Fin de chapitre </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color rgb="FFFF0000"/>
+              <sz val="9"/>
+              <scheme val="minor"/>
+            </rPr>
+            <t xml:space="preserve">à éviter 
 cf fiche de codage Insuffisance Rénale Aigue </t>
+          </r>
         </is>
       </c>
       <c r="E154" s="95" t="inlineStr">
@@ -5759,8 +6395,20 @@
       <c r="C160" s="93" t="n"/>
       <c r="D160" s="94" t="inlineStr">
         <is>
-          <t>Code de fin de chapitre 
-IMPRECIS à ne pas utiliser</t>
+          <r>
+            <t xml:space="preserve">Code de fin de chapitre 
+IMPRECIS </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color rgb="FFFF0000"/>
+              <sz val="9"/>
+              <scheme val="minor"/>
+            </rPr>
+            <t>à ne pas utiliser</t>
+          </r>
         </is>
       </c>
       <c r="E160" s="95" t="inlineStr">
@@ -5786,8 +6434,20 @@
       <c r="C161" s="93" t="n"/>
       <c r="D161" s="94" t="inlineStr">
         <is>
-          <t>Code de fin de chapitre 
-IMPRECIS à ne pas utiliser et interdit en DP</t>
+          <r>
+            <t xml:space="preserve">Code de fin de chapitre 
+IMPRECIS </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color rgb="FFFF0000"/>
+              <sz val="9"/>
+              <scheme val="minor"/>
+            </rPr>
+            <t>à ne pas utiliser et interdit en DP</t>
+          </r>
         </is>
       </c>
       <c r="E161" s="95" t="inlineStr">
@@ -5987,7 +6647,19 @@
       <c r="C169" s="1" t="n"/>
       <c r="D169" s="4" t="inlineStr">
         <is>
-          <t>Code O IMPRECIS à ne pas utiliser</t>
+          <r>
+            <t xml:space="preserve">Code O IMPRECIS </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color rgb="FFFF0000"/>
+              <sz val="9"/>
+              <scheme val="minor"/>
+            </rPr>
+            <t>à ne pas utiliser</t>
+          </r>
         </is>
       </c>
       <c r="E169" s="8" t="inlineStr">
@@ -6187,7 +6859,19 @@
       <c r="C177" s="93" t="n"/>
       <c r="D177" s="94" t="inlineStr">
         <is>
-          <t>Code O IMPRECIS à ne pas utiliser</t>
+          <r>
+            <t xml:space="preserve">Code O IMPRECIS </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color rgb="FFFF0000"/>
+              <sz val="9"/>
+              <scheme val="minor"/>
+            </rPr>
+            <t>à ne pas utiliser</t>
+          </r>
         </is>
       </c>
       <c r="E177" s="95" t="inlineStr">
@@ -6387,7 +7071,19 @@
       <c r="C185" s="93" t="n"/>
       <c r="D185" s="94" t="inlineStr">
         <is>
-          <t>Code O IMPRECIS à ne pas utiliser</t>
+          <r>
+            <t xml:space="preserve">Code O IMPRECIS </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color rgb="FFFF0000"/>
+              <sz val="9"/>
+              <scheme val="minor"/>
+            </rPr>
+            <t>à ne pas utiliser</t>
+          </r>
         </is>
       </c>
       <c r="E185" s="95" t="inlineStr">
@@ -6587,7 +7283,19 @@
       <c r="C193" s="93" t="n"/>
       <c r="D193" s="94" t="inlineStr">
         <is>
-          <t>Code O IMPRECIS à ne pas utiliser</t>
+          <r>
+            <t xml:space="preserve">Code O IMPRECIS </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color rgb="FFFF0000"/>
+              <sz val="9"/>
+              <scheme val="minor"/>
+            </rPr>
+            <t>à ne pas utiliser</t>
+          </r>
         </is>
       </c>
       <c r="E193" s="95" t="inlineStr">
@@ -6818,7 +7526,19 @@
       <c r="C202" s="93" t="n"/>
       <c r="D202" s="94" t="inlineStr">
         <is>
-          <t>Code O IMPRECIS à ne pas utiliser</t>
+          <r>
+            <t xml:space="preserve">Code O IMPRECIS </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color rgb="FFFF0000"/>
+              <sz val="9"/>
+              <scheme val="minor"/>
+            </rPr>
+            <t>à ne pas utiliser</t>
+          </r>
         </is>
       </c>
       <c r="E202" s="95" t="inlineStr">
@@ -6844,7 +7564,19 @@
       <c r="C203" s="93" t="n"/>
       <c r="D203" s="94" t="inlineStr">
         <is>
-          <t>Code O IMPRECIS à ne pas utiliser</t>
+          <r>
+            <t xml:space="preserve">Code O IMPRECIS </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color rgb="FFFF0000"/>
+              <sz val="9"/>
+              <scheme val="minor"/>
+            </rPr>
+            <t>à ne pas utiliser</t>
+          </r>
         </is>
       </c>
       <c r="E203" s="95" t="inlineStr">
@@ -7104,7 +7836,19 @@
       </c>
       <c r="D212" s="94" t="inlineStr">
         <is>
-          <t>Code O IMPRECIS à ne pas utiliser</t>
+          <r>
+            <t xml:space="preserve">Code O IMPRECIS </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color rgb="FFFF0000"/>
+              <sz val="9"/>
+              <scheme val="minor"/>
+            </rPr>
+            <t>à ne pas utiliser</t>
+          </r>
         </is>
       </c>
       <c r="E212" s="95" t="inlineStr">
@@ -7133,7 +7877,19 @@
       </c>
       <c r="D213" s="94" t="inlineStr">
         <is>
-          <t>Code O IMPRECIS à ne pas utiliser</t>
+          <r>
+            <t xml:space="preserve">Code O IMPRECIS </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color rgb="FFFF0000"/>
+              <sz val="9"/>
+              <scheme val="minor"/>
+            </rPr>
+            <t>à ne pas utiliser</t>
+          </r>
         </is>
       </c>
       <c r="E213" s="95" t="inlineStr">
@@ -7444,7 +8200,19 @@
       <c r="C225" s="93" t="n"/>
       <c r="D225" s="94" t="inlineStr">
         <is>
-          <t>Code O IMPRECIS à ne pas utiliser</t>
+          <r>
+            <t xml:space="preserve">Code O IMPRECIS </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color rgb="FFFF0000"/>
+              <sz val="9"/>
+              <scheme val="minor"/>
+            </rPr>
+            <t>à ne pas utiliser</t>
+          </r>
         </is>
       </c>
       <c r="E225" s="95" t="inlineStr">
@@ -7469,7 +8237,19 @@
       <c r="C226" s="93" t="n"/>
       <c r="D226" s="94" t="inlineStr">
         <is>
-          <t>Code O IMPRECIS à ne pas utiliser</t>
+          <r>
+            <t xml:space="preserve">Code O IMPRECIS </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color rgb="FFFF0000"/>
+              <sz val="9"/>
+              <scheme val="minor"/>
+            </rPr>
+            <t>à ne pas utiliser</t>
+          </r>
         </is>
       </c>
       <c r="E226" s="95" t="inlineStr">
@@ -9427,7 +10207,30 @@
     <row r="301">
       <c r="A301" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Insuffisance rénale aigue IRA  fonctionnelle post opératoire </t>
+          <r>
+            <t xml:space="preserve">Insuffisance rénale aigue IRA  </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="9"/>
+              <scheme val="minor"/>
+            </rPr>
+            <t>fonctionnelle</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="9"/>
+              <scheme val="minor"/>
+            </rPr>
+            <t xml:space="preserve"> post opératoire </t>
+          </r>
         </is>
       </c>
       <c r="B301" s="10" t="inlineStr">
@@ -10079,7 +10882,30 @@
     <row r="323" ht="36" customHeight="1">
       <c r="A323" s="12" t="inlineStr">
         <is>
-          <t>Extravasation d'un produit perfusé par un cathéter vasculaire sans rupture vasculaire</t>
+          <r>
+            <t xml:space="preserve">Extravasation d'un produit perfusé par un cathéter vasculaire </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="9"/>
+              <scheme val="minor"/>
+            </rPr>
+            <t>sans</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="9"/>
+              <scheme val="minor"/>
+            </rPr>
+            <t xml:space="preserve"> rupture vasculaire</t>
+          </r>
         </is>
       </c>
       <c r="B323" s="76" t="inlineStr">
@@ -10325,8 +11151,21 @@
       </c>
       <c r="F331" s="58" t="inlineStr">
         <is>
-          <t xml:space="preserve">Hématome au niveau d’une plaie obstétricale (O90.2) 
-Code en S de lésion traumatique d’un vaisseau ou bien de contusion </t>
+          <r>
+            <t xml:space="preserve">Hématome au niveau d’une plaie obstétricale (O90.2) 
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="9"/>
+              <scheme val="minor"/>
+            </rPr>
+            <t xml:space="preserve">Code en S de lésion traumatique d’un vaisseau ou bien de contusion </t>
+          </r>
         </is>
       </c>
       <c r="G331" s="6" t="n"/>
@@ -10520,7 +11359,28 @@
     <row r="338" ht="24" customHeight="1">
       <c r="A338" s="2" t="inlineStr">
         <is>
-          <t>Désunions d’une plaie opératoire non classées ailleurs, autres et non précisées (Désinsertion stomiale) (lâchage de sutures chirurgicales)</t>
+          <r>
+            <t>Désunions d’une plaie opératoire non classées ailleurs, autres et non précisées</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color rgb="FF2E74B5"/>
+              <sz val="9"/>
+              <scheme val="minor"/>
+            </rPr>
+            <t> </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <sz val="9"/>
+              <scheme val="minor"/>
+            </rPr>
+            <t>(Désinsertion stomiale) (lâchage de sutures chirurgicales)</t>
+          </r>
         </is>
       </c>
       <c r="B338" s="74" t="inlineStr">
@@ -10553,8 +11413,20 @@
     <row r="339" ht="48" customHeight="1">
       <c r="A339" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Infection après un acte à visée diagnostique et thérapeutique, non classée ailleurs (abcès , sepsis) 
-N'est pas le bon code T pour coder une infection urinaire sur sonde </t>
+          <r>
+            <t xml:space="preserve">Infection après un acte à visée diagnostique et thérapeutique, non classée ailleurs (abcès , sepsis) 
+</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color rgb="FFFF0000"/>
+              <sz val="9"/>
+              <scheme val="minor"/>
+            </rPr>
+            <t xml:space="preserve">N'est pas le bon code T pour coder une infection urinaire sur sonde </t>
+          </r>
         </is>
       </c>
       <c r="B339" s="77" t="inlineStr">
@@ -10614,7 +11486,19 @@
     <row r="341" ht="36" customHeight="1">
       <c r="A341" s="80" t="inlineStr">
         <is>
-          <t>Réaction aiguë à une substance étrangère laissée accidentellement au cours d’un acte à visée diagnostique ou thérapeutique (péritonite aseptique ou chimique)</t>
+          <r>
+            <t>R</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="9"/>
+              <scheme val="minor"/>
+            </rPr>
+            <t>éaction aiguë à une substance étrangère laissée accidentellement au cours d’un acte à visée diagnostique ou thérapeutique (péritonite aseptique ou chimique)</t>
+          </r>
         </is>
       </c>
       <c r="B341" s="79" t="inlineStr">
@@ -10670,11 +11554,42 @@
       </c>
       <c r="F342" s="81" t="inlineStr">
         <is>
-          <t xml:space="preserve">• compliquant : • avortement, grossesse extra-utérine ou molaire (O00 à O07, O08.2)
+          <r>
+            <t>•</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="9"/>
+              <scheme val="minor"/>
+            </rPr>
+            <t xml:space="preserve"> compliquant : </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Times New Roman"/>
+              <family val="1"/>
+              <color theme="1"/>
+              <sz val="9"/>
+            </rPr>
+            <t>•</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="9"/>
+              <scheme val="minor"/>
+            </rPr>
+            <t xml:space="preserve"> avortement, grossesse extra-utérine ou molaire (O00 à O07, O08.2)
 • grossesse, accouchement et puerpéralité (O88.-)
 • consécutive à une injection thérapeutique, une perfusion et une transfusion (T80.0)
 • traumatique (T79.0)
 </t>
+          </r>
         </is>
       </c>
       <c r="G342" s="6" t="inlineStr">
@@ -10920,7 +11835,30 @@
     <row r="351" ht="36" customHeight="1">
       <c r="A351" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Extravasation d'un produit perfusé par une cathéter vasculaire par rupture vasculaire (ex. erreur positionnement du cathéter , hyperdébit ou encore mauvais positionnement du bras ) </t>
+          <r>
+            <t xml:space="preserve">Extravasation d'un produit perfusé par une cathéter vasculaire par </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="9"/>
+              <scheme val="minor"/>
+            </rPr>
+            <t>rupture vasculaire</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="9"/>
+              <scheme val="minor"/>
+            </rPr>
+            <t xml:space="preserve"> (ex. erreur positionnement du cathéter , hyperdébit ou encore mauvais positionnement du bras ) </t>
+          </r>
         </is>
       </c>
       <c r="B351" s="74" t="inlineStr">
@@ -10949,7 +11887,30 @@
     <row r="352" ht="48" customHeight="1">
       <c r="A352" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Infection et réaction inflammatoire dues à une prothèse valvulaire cardiaque </t>
+          <r>
+            <t>Infection</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="9"/>
+              <scheme val="minor"/>
+            </rPr>
+            <t xml:space="preserve"> et réaction inflammatoire</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="9"/>
+              <scheme val="minor"/>
+            </rPr>
+            <t xml:space="preserve"> dues à une prothèse valvulaire cardiaque </t>
+          </r>
         </is>
       </c>
       <c r="B352" s="79" t="inlineStr">
@@ -10979,7 +11940,30 @@
     <row r="353" ht="48" customHeight="1">
       <c r="A353" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Infection et réaction inflammatoire dues à d’autres prothèses, implants et greffes cardiaques et vasculaires </t>
+          <r>
+            <t xml:space="preserve">Infection </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="9"/>
+              <scheme val="minor"/>
+            </rPr>
+            <t>et réaction inflammatoire dues</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="9"/>
+              <scheme val="minor"/>
+            </rPr>
+            <t xml:space="preserve"> à d’autres prothèses, implants et greffes cardiaques et vasculaires </t>
+          </r>
         </is>
       </c>
       <c r="B353" s="79" t="inlineStr">
@@ -27663,7 +28647,30 @@
     <row r="364" ht="36" customHeight="1">
       <c r="A364" s="12" t="inlineStr">
         <is>
-          <t>Infection et réaction inflammatoire dues à une prothèse, un implant et une greffe de l’appareil urinaire (Infection sur sonde urinaire)</t>
+          <r>
+            <t xml:space="preserve">Infection </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="9"/>
+              <scheme val="minor"/>
+            </rPr>
+            <t xml:space="preserve">et réaction inflammatoire </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="9"/>
+              <scheme val="minor"/>
+            </rPr>
+            <t>dues à une prothèse, un implant et une greffe de l’appareil urinaire (Infection sur sonde urinaire)</t>
+          </r>
         </is>
       </c>
       <c r="B364" s="79" t="inlineStr">
@@ -27673,7 +28680,36 @@
       </c>
       <c r="C364" s="4" t="inlineStr">
         <is>
-          <t>❸ SSR</t>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color rgb="FFFFC000"/>
+              <sz val="9"/>
+              <scheme val="minor"/>
+            </rPr>
+            <t>❸</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="9"/>
+              <scheme val="minor"/>
+            </rPr>
+            <t> </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color rgb="FF00B050"/>
+              <sz val="9"/>
+              <scheme val="minor"/>
+            </rPr>
+            <t>SSR</t>
+          </r>
         </is>
       </c>
       <c r="D364" s="43" t="inlineStr">
@@ -27692,7 +28728,30 @@
     <row r="365" ht="48" customHeight="1">
       <c r="A365" s="12" t="inlineStr">
         <is>
-          <t>Infection et réaction inflammatoire dues à une prothèse, un implant et une greffe de l’appareil génital</t>
+          <r>
+            <t xml:space="preserve">Infection </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="9"/>
+              <scheme val="minor"/>
+            </rPr>
+            <t xml:space="preserve">et réaction inflammatoire </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="9"/>
+              <scheme val="minor"/>
+            </rPr>
+            <t>dues à une prothèse, un implant et une greffe de l’appareil génital</t>
+          </r>
         </is>
       </c>
       <c r="B365" s="79" t="inlineStr">
@@ -27927,7 +28986,30 @@
     <row r="373" ht="48" customHeight="1">
       <c r="A373" s="12" t="inlineStr">
         <is>
-          <t>Infection et réaction inflammatoire dues à une prothèse articulaire interne</t>
+          <r>
+            <t xml:space="preserve">Infection </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="9"/>
+              <scheme val="minor"/>
+            </rPr>
+            <t>et réaction inflammatoire</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="9"/>
+              <scheme val="minor"/>
+            </rPr>
+            <t xml:space="preserve"> dues à une prothèse articulaire interne</t>
+          </r>
         </is>
       </c>
       <c r="B373" s="79" t="inlineStr">
@@ -27961,8 +29043,31 @@
     <row r="374" ht="48" customHeight="1">
       <c r="A374" s="12" t="inlineStr">
         <is>
-          <t>Infection et réaction inflammatoire dues à un appareil de fixation interne [toute localisation] 
+          <r>
+            <t xml:space="preserve">Infection </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="9"/>
+              <scheme val="minor"/>
+            </rPr>
+            <t>et réaction inflammatoire</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="9"/>
+              <scheme val="minor"/>
+            </rPr>
+            <t xml:space="preserve"> dues à un appareil de fixation interne [toute localisation] 
 ex : clou centromedullaire</t>
+          </r>
         </is>
       </c>
       <c r="B374" s="79" t="inlineStr">
@@ -27992,7 +29097,30 @@
     <row r="375" ht="48" customHeight="1">
       <c r="A375" s="12" t="inlineStr">
         <is>
-          <t>Infection et réaction inflammatoire dues à d’autres prothèses, implants et greffes orthopédiques internes</t>
+          <r>
+            <t xml:space="preserve">Infection </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="9"/>
+              <scheme val="minor"/>
+            </rPr>
+            <t xml:space="preserve">et réaction inflammatoire </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="9"/>
+              <scheme val="minor"/>
+            </rPr>
+            <t>dues à d’autres prothèses, implants et greffes orthopédiques internes</t>
+          </r>
         </is>
       </c>
       <c r="B375" s="79" t="inlineStr">
@@ -28371,7 +29499,30 @@
     <row r="389" ht="48" customHeight="1">
       <c r="A389" s="12" t="inlineStr">
         <is>
-          <t>Infection et réaction inflammatoire dues à d’autres prothèses, implants et greffes internes</t>
+          <r>
+            <t xml:space="preserve">Infection </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <b val="1"/>
+              <color theme="1"/>
+              <sz val="9"/>
+              <scheme val="minor"/>
+            </rPr>
+            <t>et réaction inflammatoire dues</t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Calibri"/>
+              <family val="2"/>
+              <color theme="1"/>
+              <sz val="9"/>
+              <scheme val="minor"/>
+            </rPr>
+            <t xml:space="preserve"> à d’autres prothèses, implants et greffes internes</t>
+          </r>
         </is>
       </c>
       <c r="B389" s="79" t="inlineStr">

</xml_diff>